<commit_message>
Venere: +3 candidati centri Milano nel funnel tracker (Corso Magenta, Via Salasco, Bocconi)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QhepYozFjjk17WbLpFAXS3
</commit_message>
<xml_diff>
--- a/Venere_Funnel_Tracker.xlsx
+++ b/Venere_Funnel_Tracker.xlsx
@@ -1072,9 +1072,21 @@
           <t>T10</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="8" t="n"/>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Corso Magenta (3 cabine + nails)</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Centro / C.so Magenta</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>idealista/ReSystems</t>
+        </is>
+      </c>
       <c r="E13" s="9" t="n"/>
       <c r="F13" s="8" t="n"/>
       <c r="G13" s="8" t="n"/>
@@ -1086,9 +1098,17 @@
       <c r="I13" s="9" t="n"/>
       <c r="J13" s="9" t="n"/>
       <c r="K13" s="9" t="n"/>
-      <c r="L13" s="8" t="n"/>
+      <c r="L13" s="8" t="inlineStr">
+        <is>
+          <t>Verificare mq (gate ambulatorio ~90mq) + reperire contatto</t>
+        </is>
+      </c>
       <c r="M13" s="9" t="n"/>
-      <c r="N13" s="8" t="n"/>
+      <c r="N13" s="8" t="inlineStr">
+        <is>
+          <t>Zona elegante, alto passaggio. 3 cabine + 5 manicure + 4 pedicure. mq da verificare. Fonte: annuncio cessione.</t>
+        </is>
+      </c>
       <c r="O13" s="8" t="n"/>
     </row>
     <row r="14">
@@ -1097,9 +1117,21 @@
           <t>T11</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="10" t="n"/>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Via Salasco (avviato)</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Porta Romana / Bocconi</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>RE/MAX</t>
+        </is>
+      </c>
       <c r="E14" s="11" t="n"/>
       <c r="F14" s="10" t="n"/>
       <c r="G14" s="10" t="n"/>
@@ -1111,9 +1143,17 @@
       <c r="I14" s="11" t="n"/>
       <c r="J14" s="11" t="n"/>
       <c r="K14" s="11" t="n"/>
-      <c r="L14" s="10" t="n"/>
+      <c r="L14" s="10" t="inlineStr">
+        <is>
+          <t>Verificare mq/dimensione + reperire contatto</t>
+        </is>
+      </c>
       <c r="M14" s="11" t="n"/>
-      <c r="N14" s="10" t="n"/>
+      <c r="N14" s="10" t="inlineStr">
+        <is>
+          <t>Avviato con clientela storica (annuncio RE/MAX). Zona vivace. Dimensione da verificare.</t>
+        </is>
+      </c>
       <c r="O14" s="10" t="n"/>
     </row>
     <row r="15">
@@ -1122,9 +1162,21 @@
           <t>T12</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="8" t="n"/>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Zona Bocconi (estetico + parrucchiere)</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Bocconi</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>portale cessione</t>
+        </is>
+      </c>
       <c r="E15" s="9" t="n"/>
       <c r="F15" s="8" t="n"/>
       <c r="G15" s="8" t="n"/>
@@ -1136,9 +1188,17 @@
       <c r="I15" s="9" t="n"/>
       <c r="J15" s="9" t="n"/>
       <c r="K15" s="9" t="n"/>
-      <c r="L15" s="8" t="n"/>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>Verificare frazionabilita in locali distinti + contatto</t>
+        </is>
+      </c>
       <c r="M15" s="9" t="n"/>
-      <c r="N15" s="8" t="n"/>
+      <c r="N15" s="8" t="inlineStr">
+        <is>
+          <t>~100 mq, alto passaggio (universita). Verificare se frazionabile per ambulatorio.</t>
+        </is>
+      </c>
       <c r="O15" s="8" t="n"/>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
Venere: arricchito Via Salasco (causa pensione, 100k) + nuovo candidato Brenta/Lodi nel tracker
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QhepYozFjjk17WbLpFAXS3
</commit_message>
<xml_diff>
--- a/Venere_Funnel_Tracker.xlsx
+++ b/Venere_Funnel_Tracker.xlsx
@@ -1119,7 +1119,7 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Via Salasco (avviato)</t>
+          <t>Via Salasco (elegante, causa pensione)</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>RE/MAX</t>
+          <t>annuncio/RE-MAX</t>
         </is>
       </c>
       <c r="E14" s="11" t="n"/>
@@ -1145,13 +1145,13 @@
       <c r="K14" s="11" t="n"/>
       <c r="L14" s="10" t="inlineStr">
         <is>
-          <t>Verificare mq/dimensione + reperire contatto</t>
+          <t>PRIORITARIO: reperire mq + contatto (venditore motivato)</t>
         </is>
       </c>
       <c r="M14" s="11" t="n"/>
       <c r="N14" s="10" t="inlineStr">
         <is>
-          <t>Avviato con clientela storica (annuncio RE/MAX). Zona vivace. Dimensione da verificare.</t>
+          <t>Causa pensione, cede a ~€100k. Clientela storica, zona elegante (Bocconi/Porta Romana). Venditore motivato. Verificare mq (gate ambulatorio).</t>
         </is>
       </c>
       <c r="O14" s="10" t="n"/>
@@ -1207,9 +1207,21 @@
           <t>T13</t>
         </is>
       </c>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="10" t="n"/>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Zona Brenta/Lodi (storico)</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Lodi / Brenta (M3)</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>annuncio</t>
+        </is>
+      </c>
       <c r="E16" s="11" t="n"/>
       <c r="F16" s="10" t="n"/>
       <c r="G16" s="10" t="n"/>
@@ -1221,9 +1233,17 @@
       <c r="I16" s="11" t="n"/>
       <c r="J16" s="11" t="n"/>
       <c r="K16" s="11" t="n"/>
-      <c r="L16" s="10" t="n"/>
+      <c r="L16" s="10" t="inlineStr">
+        <is>
+          <t>Verificare mq + bacino + contatto</t>
+        </is>
+      </c>
       <c r="M16" s="11" t="n"/>
-      <c r="N16" s="10" t="n"/>
+      <c r="N16" s="10" t="inlineStr">
+        <is>
+          <t>Centro estetico storico, clientela fidelizzata, vicino M3 Brenta. Bacino medio. Verificare dimensione.</t>
+        </is>
+      </c>
       <c r="O16" s="10" t="n"/>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Venere: arricchiti T01 Citta Studi (cessione 100k pensione, affitto) e T02 C.so Buenos Aires (bagno ATS-ready, dermopigmentazione) nel tracker
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QhepYozFjjk17WbLpFAXS3
</commit_message>
<xml_diff>
--- a/Venere_Funnel_Tracker.xlsx
+++ b/Venere_Funnel_Tracker.xlsx
@@ -661,7 +661,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>idealista/immobiliare</t>
+          <t>idealista/TrovaCasa</t>
         </is>
       </c>
       <c r="E4" s="4" t="n">
@@ -685,7 +685,7 @@
       <c r="M4" s="4" t="inlineStr"/>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>Ricavi 400k/anno, vende per pensione (venditore motivato). TOP.</t>
+          <t>Ricavi 400k/anno, cessione ~€100k causa PENSIONE (venditore motivato), canone €2.000/mese, multivetrina. Immobile in AFFITTO -&gt; verificare lease per uso sanitario + consenso opere. 100mq: verificare frazionabilita locali distinti.</t>
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr"/>
@@ -708,7 +708,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>idealista/trovacasa</t>
+          <t>Casa.it/idealista/TrovaCasa</t>
         </is>
       </c>
       <c r="E5" s="6" t="n">
@@ -732,7 +732,7 @@
       <c r="M5" s="6" t="inlineStr"/>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>110mq, bagno accessibile (ATS-friendly), zona altissimo passaggio.</t>
+          <t>110mq: 3 cabine + nails (tavolo aspirante) + reception + BAGNO SENZA BARRIERE (ATS-ready) + clima per cabina. Attivita estetica + dermopigmentazione (clientela gia para-medicale). Immobile prob. in affitto -&gt; verificare lease. Brokerata da agenzie (Casa.it/idealista/TrovaCasa).</t>
         </is>
       </c>
       <c r="O5" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Venere: Corso Buenos Aires = 75mq (sotto soglia ambulatorio), declassato a borderline/Pausa
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QhepYozFjjk17WbLpFAXS3
</commit_message>
<xml_diff>
--- a/Venere_Funnel_Tracker.xlsx
+++ b/Venere_Funnel_Tracker.xlsx
@@ -718,7 +718,7 @@
       <c r="G5" s="7" t="inlineStr"/>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>0 · Da contattare</t>
+          <t>Pausa</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
@@ -726,13 +726,13 @@
       <c r="K5" s="6" t="inlineStr"/>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>Reperire contatto + 1° messaggio</t>
+          <t>DECLASSATO: chiedere planimetria; procedere solo se il tecnico conferma layout ambulatorio a norma</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr"/>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>110mq: 3 cabine + nails (tavolo aspirante) + reception + BAGNO SENZA BARRIERE (ATS-ready) + clima per cabina. Attivita estetica + dermopigmentazione (clientela gia para-medicale). Immobile prob. in affitto -&gt; verificare lease. Brokerata da agenzie (Casa.it/idealista/TrovaCasa).</t>
+          <t>75 mq (NON 110): sotto la barra ambulatorio (~90-120). Borderline: al massimo un ambulatorio monospecialistico minimo (1 sala), da confermare con tecnico + ATS. No 2+ sale, no potenziale hub. Bagno senza barriere resta un plus. 110mq: 3 cabine + nails (tavolo aspirante) + reception + BAGNO SENZA BARRIERE (ATS-ready) + clima per cabina. Attivita estetica + dermopigmentazione (clientela gia para-medicale). Immobile prob. in affitto -&gt; verificare lease. Brokerata da agenzie (Casa.it/idealista/TrovaCasa).</t>
         </is>
       </c>
       <c r="O5" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Venere: correzione zona T01 (Viale Monza/Padova NoLo, bacino medio) + nuovo lead T14 (immobile di proprieta) + fonte B2scout
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QhepYozFjjk17WbLpFAXS3
</commit_message>
<xml_diff>
--- a/Venere_Funnel_Tracker.xlsx
+++ b/Venere_Funnel_Tracker.xlsx
@@ -656,7 +656,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Città Studi</t>
+          <t>Viale Monza/Padova (NoLo)</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -679,13 +679,13 @@
       <c r="K4" s="4" t="inlineStr"/>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>Reperire contatto titolare + 1° messaggio</t>
+          <t>Approfondire mq/frazionabilita + ticket medio clientela; priorita B (bacino medio)</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr"/>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>Ricavi 400k/anno, cessione ~€100k causa PENSIONE (venditore motivato), canone €2.000/mese, multivetrina. Immobile in AFFITTO -&gt; verificare lease per uso sanitario + consenso opere. 100mq: verificare frazionabilita locali distinti.</t>
+          <t>ZONA CORRETTA: NoLo (Viale Monza/Padova), NON Citta Studi come da annuncio -&gt; bacino MEDIO (in gentrificazione), non premium. Verificare ticket medio/reddito clientela reale. Restano positivi: 100mq, ricavi 400k, pensione, cessione 100k/affitto. Attenzione: agente ha dato zona diversa -&gt; verifica tutto.</t>
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr"/>
@@ -1252,9 +1252,21 @@
           <t>T14</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="8" t="n"/>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Centro 30+ anni con IMMOBILE DI PROPRIETA</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>da individuare</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>annuncio/B2scout</t>
+        </is>
+      </c>
       <c r="E17" s="9" t="n"/>
       <c r="F17" s="8" t="n"/>
       <c r="G17" s="8" t="n"/>
@@ -1266,9 +1278,17 @@
       <c r="I17" s="9" t="n"/>
       <c r="J17" s="9" t="n"/>
       <c r="K17" s="9" t="n"/>
-      <c r="L17" s="8" t="n"/>
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>RINTRACCIARE annuncio (idealista/B2scout): include il locale di proprieta</t>
+        </is>
+      </c>
       <c r="M17" s="9" t="n"/>
-      <c r="N17" s="8" t="n"/>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>RARO e FORTE: include il locale commerciale (PROPRIETA) -&gt; niente gate lease, consenso opere garantito, capex ambulatorio protetto. Zona e mq da individuare. Alta priorita di verifica.</t>
+        </is>
+      </c>
       <c r="O17" s="8" t="n"/>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Venere: +5 candidati online grandi/ben posizionati (Arco della Pace 140mq, Piazza Napoli, Centro 30+anni, Via Lecco 200mq, Via Nirone/Magenta)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QhepYozFjjk17WbLpFAXS3
</commit_message>
<xml_diff>
--- a/Venere_Funnel_Tracker.xlsx
+++ b/Venere_Funnel_Tracker.xlsx
@@ -1297,9 +1297,21 @@
           <t>T15</t>
         </is>
       </c>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="10" t="n"/>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Arco della Pace / Parco Sempione</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Arco della Pace (premium)</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>immobiliare/idealista</t>
+        </is>
+      </c>
       <c r="E18" s="11" t="n"/>
       <c r="F18" s="10" t="n"/>
       <c r="G18" s="10" t="n"/>
@@ -1311,9 +1323,17 @@
       <c r="I18" s="11" t="n"/>
       <c r="J18" s="11" t="n"/>
       <c r="K18" s="11" t="n"/>
-      <c r="L18" s="10" t="n"/>
+      <c r="L18" s="10" t="inlineStr">
+        <is>
+          <t>Reperire annuncio + mq/planimetria + prezzo + lease/proprieta</t>
+        </is>
+      </c>
       <c r="M18" s="11" t="n"/>
-      <c r="N18" s="10" t="n"/>
+      <c r="N18" s="10" t="inlineStr">
+        <is>
+          <t>140 mq, centro estetico OPERATIVO. Zona alto reddito/prestigio. Grande = ambulatorio comodo (2+ sale). Top candidato: verificare prezzo, lease, clientela.</t>
+        </is>
+      </c>
       <c r="O18" s="10" t="n"/>
     </row>
     <row r="19">
@@ -1322,9 +1342,21 @@
           <t>T16</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="8" t="n"/>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Piazza Napoli (ex parrucchiere+estetico)</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Piazza Napoli (semicentro W)</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>annuncio</t>
+        </is>
+      </c>
       <c r="E19" s="9" t="n"/>
       <c r="F19" s="8" t="n"/>
       <c r="G19" s="8" t="n"/>
@@ -1336,9 +1368,17 @@
       <c r="I19" s="9" t="n"/>
       <c r="J19" s="9" t="n"/>
       <c r="K19" s="9" t="n"/>
-      <c r="L19" s="8" t="n"/>
+      <c r="L19" s="8" t="inlineStr">
+        <is>
+          <t>Reperire annuncio + mq/planimetria + prezzo + lease/proprieta</t>
+        </is>
+      </c>
       <c r="M19" s="9" t="n"/>
-      <c r="N19" s="8" t="n"/>
+      <c r="N19" s="8" t="inlineStr">
+        <is>
+          <t>Dimensioni generose: 3 sale + magazzino + bagno al piano inferiore (multi-livello = ottimo per percorsi pulito/sporco). Verificare mq totali, prezzo, se attivita operativa.</t>
+        </is>
+      </c>
       <c r="O19" s="8" t="n"/>
     </row>
     <row r="20">
@@ -1347,9 +1387,21 @@
           <t>T17</t>
         </is>
       </c>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="10" t="n"/>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Centro/Piemonte 30+ anni (ZTL pedonale)</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Centro (ZTL pedonale)</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>annuncio</t>
+        </is>
+      </c>
       <c r="E20" s="11" t="n"/>
       <c r="F20" s="10" t="n"/>
       <c r="G20" s="10" t="n"/>
@@ -1361,9 +1413,17 @@
       <c r="I20" s="11" t="n"/>
       <c r="J20" s="11" t="n"/>
       <c r="K20" s="11" t="n"/>
-      <c r="L20" s="10" t="n"/>
+      <c r="L20" s="10" t="inlineStr">
+        <is>
+          <t>Reperire annuncio + mq/planimetria + prezzo + lease/proprieta</t>
+        </is>
+      </c>
       <c r="M20" s="11" t="n"/>
-      <c r="N20" s="10" t="n"/>
+      <c r="N20" s="10" t="inlineStr">
+        <is>
+          <t>Ultra-trentennale, pieno centro pedonale (zona TOP), causa TRASFERIMENTO ALL ESTERO (venditore motivato). Verificare mq + se immobile di proprieta.</t>
+        </is>
+      </c>
       <c r="O20" s="10" t="n"/>
     </row>
     <row r="21">
@@ -1372,9 +1432,21 @@
           <t>T18</t>
         </is>
       </c>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="8" t="n"/>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Via Lecco / Porta Venezia</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Porta Venezia/Lima</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Casa.it/annuncio</t>
+        </is>
+      </c>
       <c r="E21" s="9" t="n"/>
       <c r="F21" s="8" t="n"/>
       <c r="G21" s="8" t="n"/>
@@ -1386,9 +1458,17 @@
       <c r="I21" s="9" t="n"/>
       <c r="J21" s="9" t="n"/>
       <c r="K21" s="9" t="n"/>
-      <c r="L21" s="8" t="n"/>
+      <c r="L21" s="8" t="inlineStr">
+        <is>
+          <t>Reperire annuncio + mq/planimetria + prezzo + lease/proprieta</t>
+        </is>
+      </c>
       <c r="M21" s="9" t="n"/>
-      <c r="N21" s="8" t="n"/>
+      <c r="N21" s="8" t="inlineStr">
+        <is>
+          <t>~200 mq, 4 stanze + 3 bagni, 3 vetrine, zona centrale. MOLTO grande (anche hub). ATTENZIONE: verificare se e attivita operativa con clientela o solo locale/negozio vuoto.</t>
+        </is>
+      </c>
       <c r="O21" s="8" t="n"/>
     </row>
     <row r="22">
@@ -1397,9 +1477,21 @@
           <t>T19</t>
         </is>
       </c>
-      <c r="B22" s="10" t="n"/>
-      <c r="C22" s="11" t="n"/>
-      <c r="D22" s="10" t="n"/>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Via Nirone / Magenta (immobile+inquilino)</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Magenta (elegante)</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>annuncio</t>
+        </is>
+      </c>
       <c r="E22" s="11" t="n"/>
       <c r="F22" s="10" t="n"/>
       <c r="G22" s="10" t="n"/>
@@ -1411,9 +1503,17 @@
       <c r="I22" s="11" t="n"/>
       <c r="J22" s="11" t="n"/>
       <c r="K22" s="11" t="n"/>
-      <c r="L22" s="10" t="n"/>
+      <c r="L22" s="10" t="inlineStr">
+        <is>
+          <t>Reperire annuncio + mq/planimetria + prezzo + lease/proprieta</t>
+        </is>
+      </c>
       <c r="M22" s="11" t="n"/>
-      <c r="N22" s="10" t="n"/>
+      <c r="N22" s="10" t="inlineStr">
+        <is>
+          <t>Immobile commerciale con seminterrato, affittato dal 2017 a centro estetico avviato. Struttura diversa: compri l IMMOBILE con inquilino (niente gate lease per te). Zona elegante. Valutare.</t>
+        </is>
+      </c>
       <c r="O22" s="10" t="n"/>
     </row>
     <row r="23">

</xml_diff>

<commit_message>
Venere: 3 annunci idealista analizzati (Piazza Udine, Viale Umbria/Lodi, Piazza Piola/Citta Studi) - tutti senza mura, 100-110mq, convertibili
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QhepYozFjjk17WbLpFAXS3
</commit_message>
<xml_diff>
--- a/Venere_Funnel_Tracker.xlsx
+++ b/Venere_Funnel_Tracker.xlsx
@@ -651,21 +651,21 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Città Studi (multivetrina)</t>
+          <t>Piazza Udine (Pasetti, Rif 049/26)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Viale Monza/Padova (NoLo)</t>
+          <t>Piazza Udine (est, media)</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>idealista/TrovaCasa</t>
+          <t>idealista/Pasetti</t>
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>4.45</v>
+        <v>4</v>
       </c>
       <c r="F4" s="5" t="inlineStr"/>
       <c r="G4" s="5" t="inlineStr"/>
@@ -685,7 +685,7 @@
       <c r="M4" s="4" t="inlineStr"/>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>CESSIONE €90k (da telefonata). Su ricavi ~400k: se EBITDA ~15% (~60k) sono ~1,5x = molto sotto i 3-4x tipici -&gt; o AFFARE (venditore motivato) o EBITDA reale piu basso del 15% -&gt; VERIFICA i conti veri (incassi/POS). ZONA CORRETTA: NoLo (Viale Monza/Padova), NON Citta Studi come da annuncio -&gt; bacino MEDIO (in gentrificazione), non premium. Verificare ticket medio/reddito clientela reale. Restano positivi: 100mq, ricavi 400k, pensione, cessione 100k/affitto. Attenzione: agente ha dato zona diversa -&gt; verifica tutto.</t>
+          <t>SENZA MURA. 100mq, open space, 2 bagni, PIANO TERRA angolare, 7 vetrine (visibilita top). Affitto 2.000/mese, incasso 400k/anno, causa PENSIONE, cessione 90k. Pro: ricavi veri, piano terra, 2 bagni. Contro: open space da partizionare, zona media, affitto piu alto. Gate: lease+consenso opere, EBITDA reale.</t>
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr"/>
@@ -1522,10 +1522,24 @@
           <t>T20</t>
         </is>
       </c>
-      <c r="B23" s="8" t="n"/>
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="8" t="n"/>
-      <c r="E23" s="9" t="n"/>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Viale Umbria / P.le Lodi (Spampinato)</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Lodi/Viale Umbria (semicentro)</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>idealista/Spampinato</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>4.5</v>
+      </c>
       <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="n"/>
       <c r="H23" s="6" t="inlineStr">
@@ -1536,9 +1550,17 @@
       <c r="I23" s="9" t="n"/>
       <c r="J23" s="9" t="n"/>
       <c r="K23" s="9" t="n"/>
-      <c r="L23" s="8" t="n"/>
+      <c r="L23" s="8" t="inlineStr">
+        <is>
+          <t>Contattare: verificare lease (durata+consenso opere) + fatturato/EBITDA + chiarire 3 piani vs piano terra</t>
+        </is>
+      </c>
       <c r="M23" s="9" t="n"/>
-      <c r="N23" s="8" t="n"/>
+      <c r="N23" s="8" t="inlineStr">
+        <is>
+          <t>SENZA MURA. 100mq, 4 LOCALI gia divisi, 1 BAGNO DISABILI (ATS-ready), INGRESSO INDIPENDENTE (no condominio), piano terra, aria condizionata, chiavi in mano, macchinari di pregio, ottimi fatturati DIMOSTRABILI, affiancamento. 90k, affitto 1.800. TOP per conversione (minor attrito).</t>
+        </is>
+      </c>
       <c r="O23" s="8" t="n"/>
     </row>
     <row r="24">
@@ -1547,10 +1569,24 @@
           <t>T21</t>
         </is>
       </c>
-      <c r="B24" s="10" t="n"/>
-      <c r="C24" s="11" t="n"/>
-      <c r="D24" s="10" t="n"/>
-      <c r="E24" s="11" t="n"/>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Piazza Piola / V.le Romagna (Citta Studi) 110mq</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Citta Studi (media)</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>idealista</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>4.4</v>
+      </c>
       <c r="F24" s="10" t="n"/>
       <c r="G24" s="10" t="n"/>
       <c r="H24" s="4" t="inlineStr">
@@ -1561,9 +1597,17 @@
       <c r="I24" s="11" t="n"/>
       <c r="J24" s="11" t="n"/>
       <c r="K24" s="11" t="n"/>
-      <c r="L24" s="10" t="n"/>
+      <c r="L24" s="10" t="inlineStr">
+        <is>
+          <t>Contattare: lease+consenso opere + EBITDA + costo macchinari a parte</t>
+        </is>
+      </c>
       <c r="M24" s="11" t="n"/>
-      <c r="N24" s="10" t="n"/>
+      <c r="N24" s="10" t="inlineStr">
+        <is>
+          <t>SENZA MURA. 110mq (il piu grande), 3 cabine + cabina unghie (aspirazione) + reception + BAGNO SENZA BARRIERE (ATS-ready) + clima per cabina con FILTRI polveri sottili. Clientela DERMOPIGMENTAZIONE (para-medicale = miglior segnale domanda iniettabili). 99k, affitto 1.800, macchinari acquistabili a parte.</t>
+        </is>
+      </c>
       <c r="O24" s="10" t="n"/>
     </row>
     <row r="25">

</xml_diff>